<commit_message>
Fix Betül Tuncel own-course conflict and equalize Demet İrban's load
Betül Tuncel was being listed as a Saturday reserve, which overlapped
with her own TYMM Kimya exam slot (Cumartesi 09:30) — reserve
eligibility for a day now requires no own-course conflict across any
session that day, not just one. Demet İrban's artificial low-duty
handling is removed per explicit request; she now shares the normal
fair-distribution pool like everyone else.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoRQthp7m7JEvfSDqQpGzb
</commit_message>
<xml_diff>
--- a/output/Gozetmen_Programi.xlsx
+++ b/output/Gozetmen_Programi.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="C134" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="C136" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c r="C152" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="C154" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="C158" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="C160" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C162" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="C164" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -3109,7 +3109,7 @@
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C177" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="C178" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="C181" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="C182" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="C184" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="C185" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="C186" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="C187" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="C188" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C189" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="C190" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C191" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="C192" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C204" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="C205" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="C206" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="C208" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="C209" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="C210" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="C211" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3844,7 @@
       </c>
       <c r="C212" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="C213" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="C214" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="C215" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C216" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="C217" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -3946,7 +3946,7 @@
       </c>
       <c r="C218" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="C219" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -3980,7 +3980,7 @@
       </c>
       <c r="C220" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="C221" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="C234" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="C235" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4215,7 @@
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="C237" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="C238" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="C239" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="C240" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="C241" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4317,7 @@
       </c>
       <c r="C242" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="C243" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="C244" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="C245" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="C246" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="C247" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="C248" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="C249" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -4528,7 +4528,7 @@
       </c>
       <c r="C256" s="6" t="inlineStr">
         <is>
-          <t>Muhammed Karaköseoğlu</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="C257" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Muhammed Karaköseoğlu</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="C258" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="C259" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="C260" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -4613,7 +4613,7 @@
       </c>
       <c r="C261" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="C262" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="C263" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C264" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="C265" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4698,7 @@
       </c>
       <c r="C266" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4715,7 @@
       </c>
       <c r="C267" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="C268" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="C269" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="C270" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C271" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="C272" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="C273" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="C274" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="C275" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="C276" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Betül Tuncel, Sinem Kocadayı Erbiçer</t>
+          <t>Sinem Kocadayı Erbiçer, Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan, Figen Balamir</t>
+          <t>Ebru Yardım, Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -4959,7 +4959,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Ceren Tunaboylu Demir, Faruk Saylık</t>
+          <t>Emine Berrin Bostancı, Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Fatma Zeynep Saylık, Gülşah Aksungur</t>
+          <t>Ceren Tunaboylu Demir, Fatma Zeynep Saylık</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Kazım Şahin, Mehmet Ertuğrul Evyapar</t>
+          <t>Faruk Saylık, Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5102,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Demet İrban</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -5113,7 +5113,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -5124,7 +5124,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -5135,7 +5135,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -5146,7 +5146,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Faruk Saylık</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
@@ -5157,7 +5157,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Faruk Saylık</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
@@ -5168,7 +5168,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zeynep Saylık</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -5179,7 +5179,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Fatma Zeynep Saylık</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -5190,40 +5190,40 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
@@ -5234,7 +5234,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
@@ -5245,7 +5245,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
@@ -5256,7 +5256,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Muhammed Karaköseoğlu</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
@@ -5267,7 +5267,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Muhammed Karaköseoğlu</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
@@ -5278,7 +5278,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
@@ -5289,7 +5289,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
@@ -5300,7 +5300,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
@@ -5311,7 +5311,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
@@ -5322,7 +5322,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
@@ -5333,7 +5333,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
@@ -5344,7 +5344,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
@@ -5355,7 +5355,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
@@ -5366,7 +5366,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
@@ -5377,7 +5377,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
@@ -5388,7 +5388,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
@@ -5399,7 +5399,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
@@ -5410,7 +5410,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Sinem Kocadayı Erbiçer</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
       <c r="B38" s="5" t="n">
@@ -5421,7 +5421,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Sinem Kocadayı Erbiçer</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
@@ -5432,7 +5432,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
@@ -5443,7 +5443,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
@@ -5454,7 +5454,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
@@ -5465,7 +5465,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
@@ -5476,7 +5476,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
@@ -5487,7 +5487,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
@@ -5498,7 +5498,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
@@ -5509,7 +5509,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
@@ -5520,7 +5520,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
@@ -5531,7 +5531,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
       <c r="B49" s="5" t="n">
@@ -5542,22 +5542,18 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Betül Tuncel</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>Not: Yalnızca Cumartesi günü görev alabilir.</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Betül Tuncel</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
@@ -5565,7 +5561,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Not: 'Az sınav görevi' talimatı gereği en az görev.</t>
+          <t>Not: Yalnızca Cumartesi günü (kendi dersi hariç) görev alabildiği için görev sayısı düşük.</t>
         </is>
       </c>
     </row>
@@ -5634,21 +5630,21 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>6. Betül Tuncel için yalnızca Cumartesi günü (Okul Dışı Öğrenme sınavı) görev verilmiştir; kendi TYMM Kimya sınavına (Cumartesi 09:30) zaten görev verilmemiştir.</t>
+          <t>6. Betül Tuncel için yalnızca Cumartesi günü (Okul Dışı Öğrenme sınavı, saat 11:30) görev verilmiştir; kendi TYMM Kimya sınavına (Cumartesi 09:30) hiçbir şekilde görev verilmemiş, aynı sebeple Cumartesi günü yedek listesine de yazılmamıştır (o gün kendi sınavı da var).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>7. Demet İrban için 'az sınav görevi' notu gereği en az sayıda (1) görev verilmiştir.</t>
+          <t>7. Demet İrban için özel bir azaltma uygulanmamıştır; kendi dersi (Eğitim Sürecinin Yönetimi) dışında herkesle eşit şekilde görevlendirilmiştir.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>8. Her gün için en az iki yedek gözetmen belirlenmiştir (Yedekler sayfası).</t>
+          <t>8. Her gün için en az iki yedek gözetmen belirlenmiştir (Yedekler sayfası). Bir kişi, o gün kendi dersinin sınavı varsa o güne yedek olarak da yazılmamıştır.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carry each room's 09:30 proctor into the 11:30 slot of the same day
Same-day, same-room continuity: whoever proctors a room at 09:30 now
also proctors it at 11:30, unless the 11:30 exam is their own course
(then a substitute takes just that slot). Saturday keeps its earlier
Okul Dışı branch-priority pick as the anchor so that exception and this
new continuity rule both hold together; the handful of rooms where a
09:30 proctor's own course falls in the 11:30 slot (or vice versa) are
an unavoidable one-off given the fixed 24-room capacity, and are
documented in the Notlar sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoRQthp7m7JEvfSDqQpGzb
</commit_message>
<xml_diff>
--- a/output/Gozetmen_Programi.xlsx
+++ b/output/Gozetmen_Programi.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Sinem Kocadayı Erbiçer</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Sinem Kocadayı Erbiçer</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Sinem Kocadayı Erbiçer</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Sinem Kocadayı Erbiçer</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="C134" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="C136" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="C148" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c r="C152" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="C154" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="C158" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="C160" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C162" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="C164" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -3109,7 +3109,7 @@
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="C176" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C177" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="C178" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="C181" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="C182" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="C184" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="C185" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="C186" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="C187" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="C188" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C189" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="C190" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C191" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="C192" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="C201" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Sinem Kocadayı Erbiçer</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="C202" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="C203" s="6" t="inlineStr">
         <is>
-          <t>Sinem Kocadayı Erbiçer</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C204" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="C205" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="C206" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="C208" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="C209" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="C210" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="C211" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3844,7 @@
       </c>
       <c r="C212" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="C213" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="C214" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="C215" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C216" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="C217" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -3946,7 +3946,7 @@
       </c>
       <c r="C218" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="C219" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -3980,7 +3980,7 @@
       </c>
       <c r="C220" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="C221" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="C228" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zeynep Saylık</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="C229" s="6" t="inlineStr">
         <is>
-          <t>Muhammed Karaköseoğlu</t>
+          <t>Fatma Zeynep Saylık</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4113,7 @@
       </c>
       <c r="C230" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Muhammed Karaköseoğlu</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
       </c>
       <c r="C231" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="C232" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="C234" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="C235" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4215,7 @@
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="C237" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="C238" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="C239" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="C240" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="C241" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4317,7 @@
       </c>
       <c r="C242" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="C243" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="C244" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="C245" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="C246" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="C247" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="C248" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="C249" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="C255" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zeynep Saylık</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -4528,7 +4528,7 @@
       </c>
       <c r="C256" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Fatma Zeynep Saylık</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="C258" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="C259" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="C260" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -4613,7 +4613,7 @@
       </c>
       <c r="C261" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="C262" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="C263" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C264" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="C265" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4698,7 @@
       </c>
       <c r="C266" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4715,7 @@
       </c>
       <c r="C267" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="C268" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="C269" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="C270" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C271" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="C272" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="C273" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="C274" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="C275" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="C276" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Sinem Kocadayı Erbiçer, Tuba Subaşı Adıbelli</t>
+          <t>Gülşah Aksungur, Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Ebru Yardım, Emine Banu Kayhan Kırmaç</t>
+          <t>Selmi Demirkol, Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -4959,7 +4959,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı, Ezgi Sanlı</t>
+          <t>Vecihe Solmaz, Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Ceren Tunaboylu Demir, Fatma Zeynep Saylık</t>
+          <t>Sinem Kocadayı Erbiçer, Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Faruk Saylık, Fatma Zehra Çalışkan</t>
+          <t>Özkan Apaydın, Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5080,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Demet İrban</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -5091,7 +5091,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Ceren Tunaboylu Demir</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -5102,7 +5102,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -5113,7 +5113,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -5124,7 +5124,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -5135,7 +5135,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -5146,7 +5146,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
@@ -5157,7 +5157,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Faruk Saylık</t>
+          <t>Mustafa Kılıç</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
@@ -5168,7 +5168,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -5179,7 +5179,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zeynep Saylık</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -5190,7 +5190,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
@@ -5201,7 +5201,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Ceren Tunaboylu Demir</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
@@ -5212,7 +5212,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
@@ -5223,7 +5223,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
@@ -5234,7 +5234,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Faruk Saylık</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
@@ -5245,7 +5245,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
@@ -5256,7 +5256,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Fatma Zeynep Saylık</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
@@ -5267,7 +5267,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Muhammed Karaköseoğlu</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
@@ -5278,7 +5278,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
@@ -5289,7 +5289,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
@@ -5300,7 +5300,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Muhammed Karaköseoğlu</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
@@ -5311,7 +5311,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
@@ -5322,7 +5322,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
@@ -5333,7 +5333,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
@@ -5579,7 +5579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -5662,6 +5662,13 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>11. 09:30 oturumunda bir odada görevli olan kişi, aynı gün 11:30 oturumunda da (mümkünse aynı odada) görevlendirilmiştir; yalnızca 11:30 oturumu o kişinin KENDİ dersiyse, o oturuma sadece o odaya başka biri yazılmıştır. 24 odanın her ikisi de sabit kapasiteli olduğundan, bazı odalarda sabah görevlisi kendi dersi öğleden sonraya denk gelip devam edemediğinde, o odanın öğleden sonraki görevlisi (yeni kişi) sabah boş kalabilir — bu 7 oda/gün için kaçınılmaz bir istisnadır ve hiçbiri kendi dersinde görev almamıştır.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1"/>

</xml_diff>

<commit_message>
Remove Mustafa Kılıç from the proctor roster
Per request, drop him from both the room roster and daily reserves;
his slots were refilled from the fair-distribution pool.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoRQthp7m7JEvfSDqQpGzb
</commit_message>
<xml_diff>
--- a/output/Gozetmen_Programi.xlsx
+++ b/output/Gozetmen_Programi.xlsx
@@ -901,7 +901,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Sinem Kocadayı Erbiçer</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Sinem Kocadayı Erbiçer</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Sinem Kocadayı Erbiçer</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>Sinem Kocadayı Erbiçer</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="C134" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="C136" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="C148" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c r="C152" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="C154" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="C158" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="C160" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C162" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="C164" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Vecihe Solmaz</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="C176" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C177" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="C178" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="C181" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="C182" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="C184" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="C185" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="C186" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="C187" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="C188" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C189" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="C190" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C191" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="C192" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="C202" s="6" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="C203" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C204" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="C205" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Bilge Has Erdoğan</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="C206" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>Bilge Has Erdoğan</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="C208" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="C209" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
     </row>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="C210" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="C211" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3844,7 @@
       </c>
       <c r="C212" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="C213" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="C214" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="C215" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C216" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="C217" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
     </row>
@@ -3946,7 +3946,7 @@
       </c>
       <c r="C218" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Tahsin Kaya</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="C219" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -3980,7 +3980,7 @@
       </c>
       <c r="C220" s="6" t="inlineStr">
         <is>
-          <t>Tahsin Kaya</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="C221" s="6" t="inlineStr">
         <is>
-          <t>Tuba Subaşı Adıbelli</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
       </c>
       <c r="C231" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="C232" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="C234" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="C235" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4215,7 @@
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="C237" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="C238" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="C239" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="C240" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="C241" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4317,7 @@
       </c>
       <c r="C242" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="C243" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="C244" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="C245" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="C246" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="C247" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="C248" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Tuba Subaşı Adıbelli</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="C249" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="C258" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
     </row>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="C259" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="C260" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Abdullah Balcı</t>
         </is>
       </c>
     </row>
@@ -4613,7 +4613,7 @@
       </c>
       <c r="C261" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Ayşe Betül Doğruel</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="C262" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Bahar Yakut</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="C263" s="6" t="inlineStr">
         <is>
-          <t>Abdullah Balcı</t>
+          <t>Demet İrban</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C264" s="6" t="inlineStr">
         <is>
-          <t>Ayşe Betül Doğruel</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="C265" s="6" t="inlineStr">
         <is>
-          <t>Bahar Yakut</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4698,7 @@
       </c>
       <c r="C266" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4715,7 @@
       </c>
       <c r="C267" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
     </row>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="C268" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="C269" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="C270" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C271" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="C272" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="C273" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="C274" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="C275" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="C276" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur, Nuh Mustafa Beğenmez</t>
+          <t>Selmi Demirkol, Sinem Kocadayı Erbiçer</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Selmi Demirkol, Sibel Doğan</t>
+          <t>Vecihe Solmaz, Yusuf Ergül</t>
         </is>
       </c>
     </row>
@@ -4959,7 +4959,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Vecihe Solmaz, Yusuf Ergül</t>
+          <t>Zehra Gülseven, Özkan Apaydın</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Sinem Kocadayı Erbiçer, Zehra Gülseven</t>
+          <t>Bilge Has Erdoğan, Celalettin Özden</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Özkan Apaydın, Bilge Has Erdoğan</t>
+          <t>Ceren Tunaboylu Demir, Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5080,7 +5080,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Demet İrban</t>
+          <t>Celalettin Özden</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -5091,7 +5091,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Ebru Yardım</t>
+          <t>Ceren Tunaboylu Demir</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -5102,7 +5102,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Ezgi Sanlı</t>
+          <t>Demet İrban</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -5113,7 +5113,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Ertuğrul Evyapar</t>
+          <t>Ebru Yardım</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -5124,7 +5124,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Mehmet Masatoğlu</t>
+          <t>Emine Banu Kayhan Kırmaç</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -5135,7 +5135,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Mehtap Naillioğlu Kaymak</t>
+          <t>Ezgi Sanlı</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -5146,7 +5146,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Mine Bayraktar</t>
+          <t>Mehmet Ertuğrul Evyapar</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
@@ -5157,7 +5157,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Kılıç</t>
+          <t>Mehmet Masatoğlu</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
@@ -5168,7 +5168,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Nurhan Yiğit Kara</t>
+          <t>Mehtap Naillioğlu Kaymak</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -5179,7 +5179,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Sabire Ceren Demir</t>
+          <t>Mine Bayraktar</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -5190,62 +5190,62 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Celalettin Özden</t>
+          <t>Necmettin Oğuz</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Ceren Tunaboylu Demir</t>
+          <t>Nurhan Yiğit Kara</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Emine Banu Kayhan Kırmaç</t>
+          <t>Sabire Ceren Demir</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Emine Berrin Bostancı</t>
+          <t>Sibel Doğan</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Faruk Saylık</t>
+          <t>Yasemin Fatma Tekin</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zehra Çalışkan</t>
+          <t>Emine Berrin Bostancı</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
@@ -5256,7 +5256,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Fatma Zeynep Saylık</t>
+          <t>Faruk Saylık</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
@@ -5267,7 +5267,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Figen Balamir</t>
+          <t>Fatma Zehra Çalışkan</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
@@ -5278,7 +5278,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Gülşah Aksungur</t>
+          <t>Fatma Zeynep Saylık</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
@@ -5289,7 +5289,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Kazım Şahin</t>
+          <t>Figen Balamir</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
@@ -5300,7 +5300,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Muhammed Karaköseoğlu</t>
+          <t>Gülşah Aksungur</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
@@ -5311,7 +5311,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Necmettin Oğuz</t>
+          <t>Kazım Şahin</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
@@ -5322,7 +5322,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Nuh Mustafa Beğenmez</t>
+          <t>Muhammed Karaköseoğlu</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
@@ -5333,7 +5333,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Rabia Şentürk Aydın</t>
+          <t>Nuh Mustafa Beğenmez</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
@@ -5344,7 +5344,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Selmi Demirkol</t>
+          <t>Rabia Şentürk Aydın</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
@@ -5355,7 +5355,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Sema Yaniç</t>
+          <t>Selmi Demirkol</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
@@ -5366,7 +5366,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Serap Özcan</t>
+          <t>Sema Yaniç</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
@@ -5377,7 +5377,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Seval Çiğdemir</t>
+          <t>Serap Özcan</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
@@ -5388,7 +5388,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Gürses</t>
+          <t>Seval Çiğdemir</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
@@ -5399,7 +5399,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Sevgi Kırboyun</t>
+          <t>Sevgi Gürses</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
@@ -5410,7 +5410,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Sibel Doğan</t>
+          <t>Sevgi Kırboyun</t>
         </is>
       </c>
       <c r="B38" s="5" t="n">
@@ -5465,7 +5465,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Yasemin Fatma Tekin</t>
+          <t>Yavuz Gürbüz</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
@@ -5476,7 +5476,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Yavuz Gürbüz</t>
+          <t>Yunus Kütükçü</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
@@ -5487,7 +5487,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Yunus Kütükçü</t>
+          <t>Yusuf Ergül</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
@@ -5498,7 +5498,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Yusuf Ergül</t>
+          <t>Zehra Gülseven</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
@@ -5509,7 +5509,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Zehra Gülseven</t>
+          <t>Çağrı Bulut Işık</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
@@ -5520,7 +5520,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Çağrı Bulut Işık</t>
+          <t>Özkan Apaydın</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
@@ -5531,7 +5531,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Özkan Apaydın</t>
+          <t>Özlem Altınkaynak Yaylacı</t>
         </is>
       </c>
       <c r="B49" s="5" t="n">
@@ -5542,24 +5542,13 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Özlem Altınkaynak Yaylacı</t>
+          <t>Betül Tuncel</t>
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C50" s="6" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>Betül Tuncel</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>Not: Yalnızca Cumartesi günü (kendi dersi hariç) görev alabildiği için görev sayısı düşük.</t>
         </is>
@@ -5579,7 +5568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -5669,6 +5658,13 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>12. Mustafa Kılıç, kullanıcı talebi üzerine gözetmen ve yedek listesinden tamamen çıkarılmış, yerine boşalan tüm görevlere adil dağıtım havuzundan başka kişiler atanmıştır.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1"/>

</xml_diff>